<commit_message>
SEC-05 triage resolved: 78 tenant / 5 identity / 7 shared / 3 control
Apply review-item decisions:
- Integration settings (backup/vendor/telehealth) -> TENANT for the per-practice
  account/tokens; global OAuth CID/CSK stay in env/control.
- audit_logs -> TENANT (per-tenant clinical audit); super-admin auditing via a
  separate control.audit_log + break-glass/roll-up (documented).
- insurance_payers, pharmacies, laboratories, service_categories -> TENANT (per practice).

Adds an "Audit & Integration model" sheet to the triage workbook and a §10c summary
in the plan. This finalizes the tenant_tables expansion target (78 tables) for the
cutover + route sweep.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SzJ77UAHhR8QZAy3qQhqq3
</commit_message>
<xml_diff>
--- a/SEC-05_Table_Triage.xlsx
+++ b/SEC-05_Table_Triage.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Table Triage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audit &amp; Integration model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +40,12 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font/>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -55,11 +60,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -125,10 +125,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,16 +504,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SEC-05 Table Triage — tenant / identity / shared / control</t>
+          <t>SEC-05 Table Triage (resolved) — tenant / identity / shared / control</t>
         </is>
       </c>
     </row>
@@ -551,7 +557,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -561,7 +567,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -578,7 +584,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -588,7 +594,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -605,7 +611,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -615,7 +621,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -632,7 +638,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -642,7 +648,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -659,7 +665,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -669,7 +675,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -686,7 +692,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -696,7 +702,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -713,7 +719,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -723,7 +729,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -740,7 +746,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -767,7 +773,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -777,7 +783,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -794,7 +800,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -804,7 +810,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -821,7 +827,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -831,7 +837,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>GL ledger (migration 053)</t>
+          <t>GL ledger (053)</t>
         </is>
       </c>
     </row>
@@ -1026,9 +1032,9 @@
           <t>audit_logs</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>TENANT?</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1038,12 +1044,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: tenant (move) vs public+practice_id</t>
+          <t>ADD to tenant_tables + cutover</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>high-volume; PHI refs</t>
+          <t>per-tenant clinical audit; super-admin uses control.audit_log + break-glass/roll-up</t>
         </is>
       </c>
     </row>
@@ -1053,9 +1059,9 @@
           <t>backup_provider_settings</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>TENANT?</t>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1065,12 +1071,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: per-practice config vs control-plane</t>
+          <t>ADD to tenant_tables + cutover</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>integration creds</t>
+          <t>per-practice account/tokens; global CID/CSK stay in env/control</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1394,7 @@
           <t>drug_interactions</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -1573,9 +1579,9 @@
           <t>insurance_payers</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>SHARED?</t>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -1585,12 +1591,12 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: global directory vs per-practice</t>
+          <t>ADD to tenant_tables + cutover, then sweep</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>payer directory</t>
+          <t>per-practice payer list</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1613,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1617,7 +1623,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>inventory (migration 055)</t>
+          <t>inventory (055)</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1640,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1644,7 +1650,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>inventory (migration 055)</t>
+          <t>inventory (055)</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1667,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1671,7 +1677,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>inventory (migration 055)</t>
+          <t>inventory (055)</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1694,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -1715,7 +1721,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1725,7 +1731,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>inventory (migration 055)</t>
+          <t>inventory (055)</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1748,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>migration-only (not yet created?)</t>
+          <t>migration-only</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1752,7 +1758,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>inventory (migration 055)</t>
+          <t>inventory (055)</t>
         </is>
       </c>
     </row>
@@ -1785,9 +1791,9 @@
           <t>laboratories</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>SHARED?</t>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -1797,12 +1803,12 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: global directory vs per-practice</t>
+          <t>ADD to tenant_tables + cutover, then sweep</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>lab directory</t>
+          <t>per-practice lab list</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1818,7 @@
           <t>medical_codes</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -1862,7 +1868,7 @@
           <t>medication_alternatives</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -1889,7 +1895,7 @@
           <t>medications</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -2105,7 +2111,7 @@
           <t>organization_settings</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2409,7 +2415,7 @@
           <t>permissions</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -2421,7 +2427,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>keep global (no scoping)</t>
+          <t>keep global (flag: per-practice custom roles are already tenant via *_role_permissions)</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
@@ -2436,9 +2442,9 @@
           <t>pharmacies</t>
         </is>
       </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>SHARED?</t>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -2448,12 +2454,12 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: global directory vs per-practice</t>
+          <t>ADD to tenant_tables + cutover, then sweep</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>pharmacy directory</t>
+          <t>per-practice pharmacy list</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2469,7 @@
           <t>practices</t>
         </is>
       </c>
-      <c r="B77" s="7" t="inlineStr">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2586,7 +2592,7 @@
           <t>providers</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
@@ -2636,7 +2642,7 @@
           <t>role_permissions</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -2648,7 +2654,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>keep global (no scoping)</t>
+          <t>keep global (flag: per-practice custom roles are already tenant via *_role_permissions)</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -2663,7 +2669,7 @@
           <t>roles</t>
         </is>
       </c>
-      <c r="B85" s="6" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>SHARED</t>
         </is>
@@ -2675,7 +2681,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>keep global (no scoping)</t>
+          <t>keep global (flag: per-practice custom roles are already tenant via *_role_permissions)</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
@@ -2690,9 +2696,9 @@
           <t>service_categories</t>
         </is>
       </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>SHARED?</t>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -2702,12 +2708,12 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: global directory vs per-practice</t>
+          <t>ADD to tenant_tables + cutover, then sweep</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>taxonomy</t>
+          <t>per-practice taxonomy</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2723,7 @@
           <t>social_auth</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="7" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
@@ -2744,7 +2750,7 @@
           <t>subscription_plans</t>
         </is>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2794,9 +2800,9 @@
           <t>telehealth_provider_settings</t>
         </is>
       </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>TENANT?</t>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -2806,12 +2812,12 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: per-practice config vs control-plane</t>
+          <t>ADD to tenant_tables + cutover</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>integration creds</t>
+          <t>per-practice account/tokens; global CID/CSK stay in env/control</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2854,7 @@
           <t>user_role_history</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
@@ -2871,7 +2877,7 @@
           <t>user_roles</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
@@ -2894,7 +2900,7 @@
           <t>users</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
@@ -2921,9 +2927,9 @@
           <t>vendor_integration_settings</t>
         </is>
       </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>TENANT?</t>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>TENANT</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -2933,12 +2939,12 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>REVIEW: per-practice config vs control-plane</t>
+          <t>ADD to tenant_tables + cutover</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>integration creds</t>
+          <t>per-practice account/tokens; global CID/CSK stay in env/control</t>
         </is>
       </c>
     </row>
@@ -2983,17 +2989,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Resolved design decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Integration credentials (backup/vendor/telehealth)</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Global (shared)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>OAuth client id/secret (CID/CSK) live in env / control config — one app registration per provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Per-practice (tenant)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>The signed-in account, tokens, and per-practice settings live in the tenant schema (*_settings tables moved to tenant).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Audit model</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Per-tenant audit_logs</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Clinical/PHI activity, in each tenant schema. Tenant admins see only their own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>control.audit_log</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Super-admin/platform actions (tenant create/suspend, subscription changes, break-glass) — immutable, always visible to super-admin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Super-admin auditing tenant activity</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Break-glass: time-boxed, justification-required session into one tenant schema; the read itself is logged to control.audit_log. No silent cross-tenant reads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Cross-tenant reporting</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Explicit read-only roll-up that iterates tenant audit_logs (itself audited) — not a standing global view.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Classification counts</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Classification counts (resolved)</t>
         </is>
       </c>
     </row>
@@ -3004,80 +3127,53 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TENANT?</t>
+          <t>IDENTITY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IDENTITY</t>
+          <t>SHARED</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHARED</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SHARED?</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Total tables: 93</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TENANT total (incl. already-in-set) = expand tenant_tables to this set</t>
+          <t>Total: 93</t>
         </is>
       </c>
     </row>

</xml_diff>